<commit_message>
Updated Logo and code
</commit_message>
<xml_diff>
--- a/backend/dummy_students.xlsx
+++ b/backend/dummy_students.xlsx
@@ -477,7 +477,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>202511101@dau.ac.in</t>
+          <t>202511101@students.example.org</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -485,7 +485,6 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -500,7 +499,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>202511102@dau.ac.in</t>
+          <t>202511102@students.example.org</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -508,7 +507,6 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -523,7 +521,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>202511103@dau.ac.in</t>
+          <t>202511103@students.example.org</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -531,7 +529,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -546,7 +543,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>202511104@dau.ac.in</t>
+          <t>202511104@students.example.org</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -554,7 +551,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -569,7 +565,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>202511105@dau.ac.in</t>
+          <t>202511105@students.example.org</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -577,7 +573,6 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -592,7 +587,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>202511106@dau.ac.in</t>
+          <t>202511106@students.example.org</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -600,7 +595,6 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -615,7 +609,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>202511107@dau.ac.in</t>
+          <t>202511107@students.example.org</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -623,7 +617,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -638,7 +631,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>202511108@dau.ac.in</t>
+          <t>202511108@students.example.org</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -646,7 +639,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -661,7 +653,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>202511109@dau.ac.in</t>
+          <t>202511109@students.example.org</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -669,7 +661,6 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -684,7 +675,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>202511110@dau.ac.in</t>
+          <t>202511110@students.example.org</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -692,7 +683,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:E11"/>

</xml_diff>